<commit_message>
Registrar la prueba de usabilidad con tres participantes
SUS medio 74,2: RNF-15 cumplido, con la muestra reducida y la conversión
de la escala 1-10 a 1-5 declaradas en el cap. 4.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/investigacion/prueba-usabilidad-registro.xlsx
+++ b/wiki/investigacion/prueba-usabilidad-registro.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Participantes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tareas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cuestionario" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SUS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Resumen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participantes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tareas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuestionario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -63,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -72,6 +74,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,9 +454,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -559,6 +560,39 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="B2" s="5" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Belgrano, CABA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Comerciante</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>propia</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Usa X en el celular y en la computadora. SUS respondido en escala 1-10 y convertido a 1-5 (originales: 8,3,8,1,9,3,9,4,8,3).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -566,11 +600,77 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="B3" s="5" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Salta</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Odontóloga</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>propia</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Solo usa X en el celular. SUS respondido en escala 1-10 y convertido a 1-5 (originales: 9,2,7,7,7,1,8,1,7,9).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>P3</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salta</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Comerciante</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>prueba</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Casi no usa X (aprox. una vez al mes); usó una cuenta de prueba prestada. SUS respondido en escala 1-10 y convertido a 1-5 (originales: 7,3,8,7,8,3,9,3,9,10).</t>
         </is>
       </c>
     </row>
@@ -693,15 +793,45 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>sin ayuda</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Entendió sola la marca en segundos; interpretó bien colores, estados y cómo se muestra en la UI de X.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>sin ayuda</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Abrió el análisis solo en segundos. Sin dudas: al ver que las páginas de origen eran confiables, confió en el análisis.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>sin ayuda</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Abrió una fuente en segundos. Reconoció las fuentes como medios confiables (Infobae, Clarín); eso le dio confianza en el análisis.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -709,15 +839,45 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>con ayuda</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Suele usar X en el celular; en la computadora le costó, se le indicó dónde estaba la marca y la entendió fácilmente.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>con ayuda</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Por problemas de vista (usa anteojos) hubo que indicarle dónde abrir el análisis y ayudarla a leer; le costó encontrar cómo ver más información.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>sin ayuda</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Abrió sola la fuente de Infobae, el diario que lee siempre, y se puso a leerla completa.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -725,15 +885,45 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>con ayuda</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Nunca había usado X en la computadora; hubo que explicarle eso y dónde estaba la extensión. Entendió bien la marca («índice de confianza»); después quiso ir más allá para ver el detalle y la fuente.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>con ayuda</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Necesitó ayuda porque nunca usó X en la computadora. No se trabó ni hizo comentarios.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>con ayuda</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Necesitó ayuda porque no sabía usar la computadora. No se trabó; se tomó tiempo para leer la fuente completa y corroborarla con lo que decía el tweet.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -886,12 +1076,36 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Algo parecido a las notas de comunidad de X: más información sobre una publicación.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Sí, que había que hacer clic; se veía bien y se parece a las notas de comunidad de X.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Sí, son diarios argentinos conocidos y confiables; con eso supo que el veredicto era correcto.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>No, fue claro; no hay mucho para interactuar, le aparece mientras scrollea. Le resultó intuitiva.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Sí, a veces se toma más tiempo para corroborar si lo que lee es verídico en vez de scrollear de largo.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Sí, trabaja siempre en la computadora con X abierto al lado y le resulta cómodo.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -899,12 +1113,36 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>El número en verde le indicó que era algo bueno o confiable; a pesar de no ver bien, el color la ayudó a entender el estado.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Sí, después quiso indagar más sobre un posteo en particular.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Sí, vio diarios digitales que ya conoce y siempre lee, y con eso corroboró la información.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>No; solo hubo que indicarle cómo usar X en la computadora y dónde estaba la extensión. Es una nota debajo de cada posteo, nada complicado.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Un poco: ahora se toma más tiempo para detectar si algo es fake news y así informarse correctamente.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Sí, está harta de las noticias falsas, de creérselas y enterarse después de que eran falsas.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -912,12 +1150,36 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>El índice de confianza; lo entendió bien por los colores, el verde indicaba algo bueno.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Al final le quedó claro.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Sí, lo corroboró en diferentes fuentes y pudo entender que lo que vio en la noticia era verdad.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>No, porque no usaba X.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>No, porque no usa computadora.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1080,6 +1342,36 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2</v>
+      </c>
       <c r="L2">
         <f>IF(COUNT(B2:K2)=10,((B2-1)+(D2-1)+(F2-1)+(H2-1)+(J2-1)+(5-C2)+(5-E2)+(5-G2)+(5-I2)+(5-K2))*2.5,"")</f>
         <v/>
@@ -1091,6 +1383,36 @@
           <t>P2</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
       <c r="L3">
         <f>IF(COUNT(B3:K3)=10,((B3-1)+(D3-1)+(F3-1)+(H3-1)+(J3-1)+(5-C3)+(5-E3)+(5-G3)+(5-I3)+(5-K3))*2.5,"")</f>
         <v/>
@@ -1101,6 +1423,36 @@
         <is>
           <t>P3</t>
         </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5</v>
       </c>
       <c r="L4">
         <f>IF(COUNT(B4:K4)=10,((B4-1)+(D4-1)+(F4-1)+(H4-1)+(J4-1)+(5-C4)+(5-E4)+(5-G4)+(5-I4)+(5-K4))*2.5,"")</f>

</xml_diff>